<commit_message>
Add Sprint 1 presentation, user stories and test cases
</commit_message>
<xml_diff>
--- a/documents/user_stories/DUAL_User_Stories.xlsx
+++ b/documents/user_stories/DUAL_User_Stories.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="98">
   <si>
     <t>ID</t>
   </si>
@@ -36,7 +36,7 @@
     <t>Jira Key</t>
   </si>
   <si>
-    <t>Sprint 1 (22 Sep to 20 Oct): Data, model and app</t>
+    <t>Sprint 1 (22 Sep to 19 Oct): Data, model and app</t>
   </si>
   <si>
     <t>US_01</t>
@@ -222,9 +222,24 @@
     <t>SCRUM-154</t>
   </si>
   <si>
+    <t>US_18</t>
+  </si>
+  <si>
+    <t>Cloud Back End</t>
+  </si>
+  <si>
+    <t>As a screening technician, I want uploads and deletions to work reliably, so that one failed upload doesn't block the app for everyone.</t>
+  </si>
+  <si>
+    <t>A failed upload leaves no leftover file, and the next upload works. Deleting a photo never leaves the database and storage out of sync. The API tests run against a separate test database (never the shared one) and pass, including the PDF exports. Anyone can set up the back end from the repo using the schema, .env.example and README. The docs and diagrams describe Supabase, not SQLite.</t>
+  </si>
+  <si>
     <t>Sprint 3 (planned)</t>
   </si>
   <si>
+    <t>SCRUM-62</t>
+  </si>
+  <si>
     <t>US_12</t>
   </si>
   <si>
@@ -237,7 +252,7 @@
     <t>Grad-CAM heatmaps are produced for ORIGA and DRISHTI-GS; the share of images whose heatmap peak falls inside the disc outline is reported per dataset.</t>
   </si>
   <si>
-    <t>SCRUM-62</t>
+    <t>SCRUM-63</t>
   </si>
   <si>
     <t>US_13</t>
@@ -252,7 +267,7 @@
     <t>Single-disease and shared models are compared per disease on the internal test and, for glaucoma, on the external tests; spread across seeds is shown; table and conclusion are in the repository.</t>
   </si>
   <si>
-    <t>SCRUM-63</t>
+    <t>SCRUM-64</t>
   </si>
   <si>
     <t>US_14</t>
@@ -267,7 +282,7 @@
     <t>The app runs on the trained model; "Uncertain, refer" is shown as a normal result; every results table names the commit that produced it; the results commit is tagged before the final demo.</t>
   </si>
   <si>
-    <t>SCRUM-64</t>
+    <t>SCRUM-65</t>
   </si>
   <si>
     <t>US_15</t>
@@ -282,7 +297,7 @@
     <t>Data card, user manual, deployment manual and API documentation in PDF and Word; final technical paper with its history page; reviewed by the data pipeline and external validation roles.</t>
   </si>
   <si>
-    <t>SCRUM-65</t>
+    <t>SCRUM-156</t>
   </si>
   <si>
     <t>US_17</t>
@@ -292,9 +307,6 @@
   </si>
   <si>
     <t>Test cases are written for each Sprint 3 story; each is run and recorded as pass or fail with the date; the full app is tested end to end with the real model before the final demo; every pull request is reviewed before it is merged; problems found are logged in Jira.</t>
-  </si>
-  <si>
-    <t>SCRUM-156</t>
   </si>
   <si>
     <t>Total</t>
@@ -319,7 +331,7 @@
     </font>
     <font>
       <b/>
-      <sz val="10.0"/>
+      <sz val="11.0"/>
       <color rgb="FF2A63C9"/>
       <name val="Montserrat"/>
     </font>
@@ -331,12 +343,12 @@
     </font>
     <font>
       <b/>
-      <sz val="10.0"/>
+      <sz val="11.0"/>
       <color rgb="FF36353C"/>
       <name val="Montserrat"/>
     </font>
     <font>
-      <sz val="10.0"/>
+      <sz val="11.0"/>
       <color rgb="FF36353C"/>
       <name val="Montserrat"/>
     </font>
@@ -422,28 +434,33 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="20">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="2" fillId="3" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
+    <xf borderId="2" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment vertical="bottom"/>
+    </xf>
     <xf borderId="3" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="1" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="bottom"/>
     </xf>
     <xf borderId="1" fillId="3" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
     <xf borderId="1" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="top" wrapText="1"/>
+      <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="top" wrapText="1"/>
+      <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="top" wrapText="1"/>
@@ -451,11 +468,23 @@
     <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="right"/>
+    <xf borderId="2" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment vertical="bottom"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="right" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" vertical="bottom"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyFont="1"/>
   </cellXfs>
@@ -696,401 +725,420 @@
       <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="2" ht="21.75" customHeight="1">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="6">
+      <c r="B2" s="5"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="7">
         <f>SUM(E3:E8)</f>
         <v>83</v>
       </c>
-      <c r="F2" s="7"/>
+      <c r="F2" s="8"/>
     </row>
     <row r="3" ht="63.0" customHeight="1">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="C3" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="D3" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="10">
+      <c r="E3" s="11">
         <v>23.0</v>
       </c>
-      <c r="F3" s="11" t="s">
+      <c r="F3" s="12" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="4" ht="57.0" customHeight="1">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="C4" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="D4" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="10">
+      <c r="E4" s="11">
         <v>16.0</v>
       </c>
-      <c r="F4" s="11" t="s">
+      <c r="F4" s="12" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="5" ht="63.0" customHeight="1">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="C5" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="D5" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="E5" s="10">
+      <c r="E5" s="11">
         <v>15.0</v>
       </c>
-      <c r="F5" s="11" t="s">
+      <c r="F5" s="12" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="6" ht="62.25" customHeight="1">
-      <c r="A6" s="8" t="s">
+    <row r="6" ht="86.25" customHeight="1">
+      <c r="A6" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="C6" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="D6" s="9" t="s">
+      <c r="D6" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="E6" s="10">
+      <c r="E6" s="11">
         <v>18.0</v>
       </c>
-      <c r="F6" s="11" t="s">
+      <c r="F6" s="12" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="7" ht="54.75" customHeight="1">
-      <c r="A7" s="8" t="s">
+    <row r="7" ht="61.5" customHeight="1">
+      <c r="A7" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="C7" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="D7" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="10">
+      <c r="E7" s="11">
         <v>3.0</v>
       </c>
-      <c r="F7" s="11" t="s">
+      <c r="F7" s="12" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="8" ht="61.5" customHeight="1">
-      <c r="A8" s="8" t="s">
+      <c r="A8" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="C8" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="D8" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="E8" s="10">
+      <c r="E8" s="11">
         <v>8.0</v>
       </c>
-      <c r="F8" s="11" t="s">
+      <c r="F8" s="12" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="9" ht="21.75" customHeight="1">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="B9" s="4"/>
-      <c r="C9" s="4"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="6">
-        <f>SUM(E10:E15)</f>
-        <v>28</v>
-      </c>
-      <c r="F9" s="7"/>
+      <c r="B9" s="5"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="6"/>
+      <c r="E9" s="7">
+        <f>SUM(E10:E16)</f>
+        <v>36</v>
+      </c>
+      <c r="F9" s="8"/>
     </row>
     <row r="10" ht="54.75" customHeight="1">
-      <c r="A10" s="8" t="s">
+      <c r="A10" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="B10" s="9" t="s">
+      <c r="B10" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="C10" s="9" t="s">
+      <c r="C10" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="D10" s="9" t="s">
+      <c r="D10" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="E10" s="10">
+      <c r="E10" s="11">
         <v>5.0</v>
       </c>
-      <c r="F10" s="11" t="s">
+      <c r="F10" s="12" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="11" ht="48.75" customHeight="1">
-      <c r="A11" s="8" t="s">
+      <c r="A11" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="B11" s="9" t="s">
+      <c r="B11" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="C11" s="9" t="s">
+      <c r="C11" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="D11" s="9" t="s">
+      <c r="D11" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="E11" s="10">
+      <c r="E11" s="11">
         <v>3.0</v>
       </c>
-      <c r="F11" s="11" t="s">
+      <c r="F11" s="12" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="12" ht="58.5" customHeight="1">
-      <c r="A12" s="8" t="s">
+      <c r="A12" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="B12" s="9" t="s">
+      <c r="B12" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="C12" s="9" t="s">
+      <c r="C12" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="D12" s="9" t="s">
+      <c r="D12" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="E12" s="10">
+      <c r="E12" s="11">
         <v>5.0</v>
       </c>
-      <c r="F12" s="11" t="s">
+      <c r="F12" s="12" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="13" ht="50.25" customHeight="1">
-      <c r="A13" s="8" t="s">
+    <row r="13" ht="57.75" customHeight="1">
+      <c r="A13" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="B13" s="9" t="s">
+      <c r="B13" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="C13" s="9" t="s">
+      <c r="C13" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="D13" s="9" t="s">
+      <c r="D13" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="E13" s="10">
+      <c r="E13" s="11">
         <v>5.0</v>
       </c>
-      <c r="F13" s="11" t="s">
+      <c r="F13" s="12" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="14" ht="58.5" customHeight="1">
-      <c r="A14" s="8" t="s">
+      <c r="A14" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="B14" s="9" t="s">
+      <c r="B14" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="C14" s="9" t="s">
+      <c r="C14" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="D14" s="9" t="s">
+      <c r="D14" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="E14" s="10">
+      <c r="E14" s="11">
         <v>5.0</v>
       </c>
-      <c r="F14" s="11" t="s">
+      <c r="F14" s="12" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="15" ht="57.0" customHeight="1">
-      <c r="A15" s="8" t="s">
+    <row r="15" ht="66.0" customHeight="1">
+      <c r="A15" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="B15" s="9" t="s">
+      <c r="B15" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="C15" s="9" t="s">
+      <c r="C15" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="D15" s="9" t="s">
+      <c r="D15" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="E15" s="10">
+      <c r="E15" s="11">
         <v>5.0</v>
       </c>
-      <c r="F15" s="11" t="s">
+      <c r="F15" s="12" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="16" ht="21.75" customHeight="1">
-      <c r="A16" s="3" t="s">
+    <row r="16" ht="112.5" customHeight="1">
+      <c r="A16" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="B16" s="4"/>
-      <c r="C16" s="4"/>
-      <c r="D16" s="5"/>
-      <c r="E16" s="6">
-        <f>SUM(E17:E21)</f>
+      <c r="B16" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="C16" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="D16" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="E16" s="11">
+        <v>8.0</v>
+      </c>
+      <c r="F16" s="8"/>
+    </row>
+    <row r="17" ht="27.0" customHeight="1">
+      <c r="A17" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="B17" s="5"/>
+      <c r="C17" s="5"/>
+      <c r="D17" s="6"/>
+      <c r="E17" s="7">
+        <f>SUM(E18:E22)</f>
         <v>29</v>
       </c>
-      <c r="F16" s="7"/>
-    </row>
-    <row r="17" ht="50.25" customHeight="1">
-      <c r="A17" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="B17" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="C17" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="D17" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="E17" s="10">
+      <c r="F17" s="12" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="18" ht="57.75" customHeight="1">
+      <c r="A18" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="B18" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="C18" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="D18" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="E18" s="11">
         <v>5.0</v>
       </c>
-      <c r="F17" s="11" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="18" ht="57.75" customHeight="1">
-      <c r="A18" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="B18" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="C18" s="9" t="s">
-        <v>76</v>
-      </c>
-      <c r="D18" s="9" t="s">
-        <v>77</v>
-      </c>
-      <c r="E18" s="10">
+      <c r="F18" s="12" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="19" ht="55.5" customHeight="1">
+      <c r="A19" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="B19" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="C19" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="D19" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="E19" s="11">
         <v>3.0</v>
       </c>
-      <c r="F18" s="11" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="19" ht="55.5" customHeight="1">
-      <c r="A19" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="B19" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="C19" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="D19" s="9" t="s">
-        <v>82</v>
-      </c>
-      <c r="E19" s="10">
+      <c r="F19" s="12" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="20" ht="57.0" customHeight="1">
+      <c r="A20" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="B20" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="C20" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="D20" s="10" t="s">
+        <v>87</v>
+      </c>
+      <c r="E20" s="11">
         <v>8.0</v>
       </c>
-      <c r="F19" s="11" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="20" ht="57.0" customHeight="1">
-      <c r="A20" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="B20" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="C20" s="9" t="s">
-        <v>86</v>
-      </c>
-      <c r="D20" s="9" t="s">
-        <v>87</v>
-      </c>
-      <c r="E20" s="10">
+      <c r="F20" s="12" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="21" ht="71.25" customHeight="1">
+      <c r="A21" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="B21" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="C21" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="D21" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="E21" s="11">
         <v>8.0</v>
       </c>
-      <c r="F20" s="11" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="21" ht="71.25" customHeight="1">
-      <c r="A21" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="B21" s="9" t="s">
+      <c r="F21" s="12" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="22" ht="75.75" customHeight="1">
+      <c r="A22" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="B22" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="C21" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="D21" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="E21" s="10">
+      <c r="C22" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="D22" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="E22" s="11">
         <v>5.0</v>
       </c>
-      <c r="F21" s="11" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="22" ht="15.75" customHeight="1">
-      <c r="D22" s="12" t="s">
-        <v>93</v>
-      </c>
-      <c r="E22" s="13">
-        <f>E2+E9+E16</f>
-        <v>140</v>
-      </c>
-    </row>
-    <row r="23" ht="15.75" customHeight="1"/>
+    </row>
+    <row r="23" ht="15.75" customHeight="1">
+      <c r="A23" s="16"/>
+      <c r="B23" s="16"/>
+      <c r="C23" s="16"/>
+      <c r="D23" s="17" t="s">
+        <v>97</v>
+      </c>
+      <c r="E23" s="18">
+        <f>E2+E9+E17</f>
+        <v>148</v>
+      </c>
+    </row>
     <row r="24" ht="15.75" customHeight="1">
-      <c r="A24" s="14"/>
+      <c r="A24" s="19"/>
     </row>
     <row r="25" ht="15.75" customHeight="1"/>
     <row r="26" ht="15.75" customHeight="1"/>
@@ -2072,7 +2120,7 @@
   <mergeCells count="3">
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A9:D9"/>
-    <mergeCell ref="A16:D16"/>
+    <mergeCell ref="A17:D17"/>
   </mergeCells>
   <printOptions/>
   <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>

</xml_diff>